<commit_message>
Import lại hiển thị process %
</commit_message>
<xml_diff>
--- a/import-so-TMDT.xlsx
+++ b/import-so-TMDT.xlsx
@@ -54,9 +54,6 @@
     <t>Ghi chú</t>
   </si>
   <si>
-    <t>0788.812.3456</t>
-  </si>
-  <si>
     <t>Sim sánh tiến</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>Đang giao</t>
   </si>
   <si>
-    <t>0788.812.3460</t>
-  </si>
-  <si>
     <t>Sim dễ nhớ</t>
   </si>
   <si>
@@ -90,12 +84,6 @@
     <t>Đã đăng bán</t>
   </si>
   <si>
-    <t>07888123456</t>
-  </si>
-  <si>
-    <t>07888123460</t>
-  </si>
-  <si>
     <t>Cọc sim</t>
   </si>
   <si>
@@ -109,6 +97,18 @@
   </si>
   <si>
     <t>DH2</t>
+  </si>
+  <si>
+    <t>07888123466</t>
+  </si>
+  <si>
+    <t>07888123455</t>
+  </si>
+  <si>
+    <t>0788.812.3455</t>
+  </si>
+  <si>
+    <t>0788.812.3466</t>
   </si>
 </sst>
 </file>
@@ -462,7 +462,7 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -477,7 +477,7 @@
         <v>9</v>
       </c>
       <c r="L1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>10</v>
@@ -488,37 +488,37 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" t="s">
-        <v>17</v>
-      </c>
       <c r="L2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -526,37 +526,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
       </c>
       <c r="I3" s="2">
         <v>25324</v>
       </c>
       <c r="J3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>